<commit_message>
data: WM W28 other_channels sales update (operator edit)
Operator updated data/raw/sales/Week 28/White_Mulberry/other_channels.xlsx
with additional/corrected sales rows.  Push triggers Weekly Auto-Sync
via path filter (data/raw/sales/**) which will re-run business_report_derive
-> sales_auto_etl -> step4 -> step5 and regenerate all snapshots on CI.

The step4 notna() fix (1ec0182) is in place so the regen will produce
clean output and the brand-mistag gate will pass.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/raw/sales/Week 28/White_Mulberry/other_channels.xlsx
+++ b/data/raw/sales/Week 28/White_Mulberry/other_channels.xlsx
@@ -5,15 +5,15 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Hazique Backup\Week 17\Week 28\raw\sales\Week 28\White_Mulberry\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Other computers\My Laptop\D\Nitesh\Weekly Report - B2B + B2C\FastAPI\data\raw\sales\Week 28\White_Mulberry\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98E08A04-7F2D-4643-9422-59C5E149B10E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{881D24C2-94F7-49C0-A22D-4FB1C23A307D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="4" r:id="rId1"/>
+    <sheet name="1p Sales" sheetId="4" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="22">
   <si>
     <t>ASIN</t>
   </si>
@@ -97,36 +97,15 @@
   </si>
   <si>
     <t>White Mulberry</t>
-  </si>
-  <si>
-    <t>₹1,68,049.77</t>
-  </si>
-  <si>
-    <t>₹1,05,717.11</t>
-  </si>
-  <si>
-    <t>₹44,210.04</t>
-  </si>
-  <si>
-    <t>₹38,390.04</t>
-  </si>
-  <si>
-    <t>₹26,687.29</t>
-  </si>
-  <si>
-    <t>₹24,633.91</t>
-  </si>
-  <si>
-    <t>₹5,505.09</t>
-  </si>
-  <si>
-    <t>₹0.00</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="8" formatCode="&quot;₹&quot;\ #,##0.00;[Red]&quot;₹&quot;\ \-#,##0.00"/>
+  </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -155,8 +134,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -402,11 +382,11 @@
       <c r="C2" t="s">
         <v>21</v>
       </c>
-      <c r="D2" t="s">
-        <v>22</v>
+      <c r="D2" s="1">
+        <v>175038.75</v>
       </c>
       <c r="E2">
-        <v>76</v>
+        <v>79</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
@@ -419,11 +399,11 @@
       <c r="C3" t="s">
         <v>21</v>
       </c>
-      <c r="D3" t="s">
-        <v>23</v>
+      <c r="D3" s="1">
+        <v>110799.31</v>
       </c>
       <c r="E3">
-        <v>64</v>
+        <v>67</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
@@ -436,11 +416,11 @@
       <c r="C4" t="s">
         <v>21</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="1">
+        <v>62593.97</v>
+      </c>
+      <c r="E4">
         <v>24</v>
-      </c>
-      <c r="E4">
-        <v>17</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
@@ -453,11 +433,11 @@
       <c r="C5" t="s">
         <v>21</v>
       </c>
-      <c r="D5" t="s">
-        <v>25</v>
+      <c r="D5" s="1">
+        <v>43472.25</v>
       </c>
       <c r="E5">
-        <v>23</v>
+        <v>26</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
@@ -470,8 +450,8 @@
       <c r="C6" t="s">
         <v>21</v>
       </c>
-      <c r="D6" t="s">
-        <v>26</v>
+      <c r="D6" s="1">
+        <v>26687.29</v>
       </c>
       <c r="E6">
         <v>9</v>
@@ -487,8 +467,8 @@
       <c r="C7" t="s">
         <v>21</v>
       </c>
-      <c r="D7" t="s">
-        <v>27</v>
+      <c r="D7" s="1">
+        <v>24633.91</v>
       </c>
       <c r="E7">
         <v>7</v>
@@ -504,11 +484,11 @@
       <c r="C8" t="s">
         <v>21</v>
       </c>
-      <c r="D8" t="s">
-        <v>28</v>
+      <c r="D8" s="1">
+        <v>4107.63</v>
       </c>
       <c r="E8">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
@@ -521,8 +501,8 @@
       <c r="C9" t="s">
         <v>21</v>
       </c>
-      <c r="D9" t="s">
-        <v>29</v>
+      <c r="D9" s="1">
+        <v>0</v>
       </c>
       <c r="E9">
         <v>0</v>

</xml_diff>